<commit_message>
Add Universal Knowledge Graph Builder mode for arbitrary Excel sheets, dynamic entity color palettes, and multi-domain sample datasets
</commit_message>
<xml_diff>
--- a/sampleData/enterprise_application_stack.xlsx
+++ b/sampleData/enterprise_application_stack.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Application Portfolio" sheetId="1" r:id="rId1"/>
+    <sheet name="Applications" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -397,21 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L21"/>
-  <cols>
-    <col min="1" max="1" width="30.83203125" customWidth="1"/>
-    <col min="2" max="2" width="25.83203125" customWidth="1"/>
-    <col min="3" max="3" width="20.83203125" customWidth="1"/>
-    <col min="4" max="4" width="24.83203125" customWidth="1"/>
-    <col min="5" max="5" width="20.83203125" customWidth="1"/>
-    <col min="6" max="6" width="25.83203125" customWidth="1"/>
-    <col min="7" max="7" width="35.83203125" customWidth="1"/>
-    <col min="8" max="8" width="22.83203125" customWidth="1"/>
-    <col min="9" max="9" width="15.83203125" customWidth="1"/>
-    <col min="10" max="10" width="20.83203125" customWidth="1"/>
-    <col min="11" max="11" width="35.83203125" customWidth="1"/>
-    <col min="12" max="12" width="60.83203125" customWidth="1"/>
-  </cols>
+  <dimension ref="A1:L11"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -831,389 +817,9 @@
         <v>Historical email and memo repository kept alive strictly for compliance retention. Only queried 2-3 times per year.</v>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" t="str">
-        <v>Tableau Analytics Server</v>
-      </c>
-      <c r="B12" t="str">
-        <v>Analytics &amp; BI</v>
-      </c>
-      <c r="C12" t="str">
-        <v>Medium</v>
-      </c>
-      <c r="D12">
-        <v>260000</v>
-      </c>
-      <c r="E12" t="str">
-        <v>Stable</v>
-      </c>
-      <c r="F12" t="str">
-        <v>On-Premises VM</v>
-      </c>
-      <c r="G12" t="str">
-        <v>Tableau Server, PostgreSQL, Windows Server</v>
-      </c>
-      <c r="H12" t="str">
-        <v>Cloud Ready</v>
-      </c>
-      <c r="I12">
-        <v>1100</v>
-      </c>
-      <c r="J12" t="str">
-        <v>Salesforce / Tableau</v>
-      </c>
-      <c r="K12" t="str">
-        <v>Snowflake Data Warehouse</v>
-      </c>
-      <c r="L12" t="str">
-        <v>On-prem dashboard server. High infrastructure cost compared to Tableau Cloud or Power BI embedded.</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="str">
-        <v>Legacy FoxPro Inventory</v>
-      </c>
-      <c r="B13" t="str">
-        <v>Supply Chain &amp; Logistics</v>
-      </c>
-      <c r="C13" t="str">
-        <v>Low</v>
-      </c>
-      <c r="D13">
-        <v>95000</v>
-      </c>
-      <c r="E13" t="str">
-        <v>EOL &amp; Fragile</v>
-      </c>
-      <c r="F13" t="str">
-        <v>Local Windows Server 2008</v>
-      </c>
-      <c r="G13" t="str">
-        <v>Visual FoxPro 9.0, DBF files</v>
-      </c>
-      <c r="H13" t="str">
-        <v>Legacy Incompatible</v>
-      </c>
-      <c r="I13">
-        <v>12</v>
-      </c>
-      <c r="J13" t="str">
-        <v>In-House</v>
-      </c>
-      <c r="K13" t="str">
-        <v>Oracle E-Business Suite 11i</v>
-      </c>
-      <c r="L13" t="str">
-        <v>Regional warehouse stock tracker run on an unpatched Windows 2008 machine. Severe single-point-of-failure.</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="str">
-        <v>Jira &amp; Confluence Cloud</v>
-      </c>
-      <c r="B14" t="str">
-        <v>Engineering</v>
-      </c>
-      <c r="C14" t="str">
-        <v>High</v>
-      </c>
-      <c r="D14">
-        <v>175000</v>
-      </c>
-      <c r="E14" t="str">
-        <v>Modern SaaS</v>
-      </c>
-      <c r="F14" t="str">
-        <v>SaaS</v>
-      </c>
-      <c r="G14" t="str">
-        <v>Atlassian Cloud REST API, Forge</v>
-      </c>
-      <c r="H14" t="str">
-        <v>Cloud Native</v>
-      </c>
-      <c r="I14">
-        <v>1400</v>
-      </c>
-      <c r="J14" t="str">
-        <v>Atlassian</v>
-      </c>
-      <c r="K14" t="str">
-        <v>Active Directory</v>
-      </c>
-      <c r="L14" t="str">
-        <v>Standardized issue tracking, product sprint planning, and engineering knowledge base.</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="str">
-        <v>ServiceNow ITOM</v>
-      </c>
-      <c r="B15" t="str">
-        <v>IT Infrastructure</v>
-      </c>
-      <c r="C15" t="str">
-        <v>High</v>
-      </c>
-      <c r="D15">
-        <v>390000</v>
-      </c>
-      <c r="E15" t="str">
-        <v>Modern SaaS</v>
-      </c>
-      <c r="F15" t="str">
-        <v>SaaS</v>
-      </c>
-      <c r="G15" t="str">
-        <v>ServiceNow Now Platform, JavaScript</v>
-      </c>
-      <c r="H15" t="str">
-        <v>Cloud Native</v>
-      </c>
-      <c r="I15">
-        <v>2200</v>
-      </c>
-      <c r="J15" t="str">
-        <v>ServiceNow</v>
-      </c>
-      <c r="K15" t="str">
-        <v>Active Directory, Jira &amp; Confluence Cloud</v>
-      </c>
-      <c r="L15" t="str">
-        <v>IT service desk, incident response, CMDB configuration management, and change approvals.</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="str">
-        <v>Custom C# WinForms POS</v>
-      </c>
-      <c r="B16" t="str">
-        <v>Retail Operations</v>
-      </c>
-      <c r="C16" t="str">
-        <v>High</v>
-      </c>
-      <c r="D16">
-        <v>340000</v>
-      </c>
-      <c r="E16" t="str">
-        <v>High Tech Debt</v>
-      </c>
-      <c r="F16" t="str">
-        <v>On-Premises Store PCs</v>
-      </c>
-      <c r="G16" t="str">
-        <v>.NET Framework 3.5, C#, SQL Server Express</v>
-      </c>
-      <c r="H16" t="str">
-        <v>Monolith Heavy</v>
-      </c>
-      <c r="I16">
-        <v>850</v>
-      </c>
-      <c r="J16" t="str">
-        <v>In-House</v>
-      </c>
-      <c r="K16" t="str">
-        <v>Legacy AS400 Core Banking</v>
-      </c>
-      <c r="L16" t="str">
-        <v>In-store desktop point-of-sale software requiring manual onsite updates across 120 retail branches.</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="str">
-        <v>CyberArk Privileged Access Vault</v>
-      </c>
-      <c r="B17" t="str">
-        <v>IT Security</v>
-      </c>
-      <c r="C17" t="str">
-        <v>Mission Critical</v>
-      </c>
-      <c r="D17">
-        <v>210000</v>
-      </c>
-      <c r="E17" t="str">
-        <v>Modern</v>
-      </c>
-      <c r="F17" t="str">
-        <v>Hybrid Cloud</v>
-      </c>
-      <c r="G17" t="str">
-        <v>CyberArk EPV, Vault Protocol, REST API</v>
-      </c>
-      <c r="H17" t="str">
-        <v>Cloud Ready</v>
-      </c>
-      <c r="I17">
-        <v>350</v>
-      </c>
-      <c r="J17" t="str">
-        <v>CyberArk</v>
-      </c>
-      <c r="K17" t="str">
-        <v>Active Directory</v>
-      </c>
-      <c r="L17" t="str">
-        <v>Enterprise credential rotation, SSH key management, and zero-trust privileged account access enforcement.</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="str">
-        <v>Legacy Perl Report Generator</v>
-      </c>
-      <c r="B18" t="str">
-        <v>Finance &amp; Accounting</v>
-      </c>
-      <c r="C18" t="str">
-        <v>Low</v>
-      </c>
-      <c r="D18">
-        <v>75000</v>
-      </c>
-      <c r="E18" t="str">
-        <v>EOL &amp; Fragile</v>
-      </c>
-      <c r="F18" t="str">
-        <v>Linux Server</v>
-      </c>
-      <c r="G18" t="str">
-        <v>Perl 5.10, Flat Files, Cron</v>
-      </c>
-      <c r="H18" t="str">
-        <v>Legacy Incompatible</v>
-      </c>
-      <c r="I18">
-        <v>4</v>
-      </c>
-      <c r="J18" t="str">
-        <v>In-House</v>
-      </c>
-      <c r="K18" t="str">
-        <v>Legacy AS400 Core Banking, SAP S/4HANA Finance</v>
-      </c>
-      <c r="L18" t="str">
-        <v>Nightly reconciliation script written by a former employee in 2006. Unmaintained and breaks on leap years.</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="str">
-        <v>Datadog Cloud Observability</v>
-      </c>
-      <c r="B19" t="str">
-        <v>Engineering</v>
-      </c>
-      <c r="C19" t="str">
-        <v>High</v>
-      </c>
-      <c r="D19">
-        <v>290000</v>
-      </c>
-      <c r="E19" t="str">
-        <v>Modern SaaS</v>
-      </c>
-      <c r="F19" t="str">
-        <v>SaaS</v>
-      </c>
-      <c r="G19" t="str">
-        <v>Datadog Agent, OpenTelemetry, APM</v>
-      </c>
-      <c r="H19" t="str">
-        <v>Cloud Native</v>
-      </c>
-      <c r="I19">
-        <v>450</v>
-      </c>
-      <c r="J19" t="str">
-        <v>Datadog</v>
-      </c>
-      <c r="K19" t="str">
-        <v>Custom Python Microservices, AWS Cloud Infrastructure</v>
-      </c>
-      <c r="L19" t="str">
-        <v>Unified distributed tracing, synthetic checks, log aggregation, and real-time infrastructure alerting.</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="str">
-        <v>Active Directory &amp; Entra ID</v>
-      </c>
-      <c r="B20" t="str">
-        <v>IT Infrastructure</v>
-      </c>
-      <c r="C20" t="str">
-        <v>Mission Critical</v>
-      </c>
-      <c r="D20">
-        <v>180000</v>
-      </c>
-      <c r="E20" t="str">
-        <v>Modern</v>
-      </c>
-      <c r="F20" t="str">
-        <v>Hybrid Cloud</v>
-      </c>
-      <c r="G20" t="str">
-        <v>SAML 2.0, OIDC, Kerberos, Azure AD</v>
-      </c>
-      <c r="H20" t="str">
-        <v>Cloud Native</v>
-      </c>
-      <c r="I20">
-        <v>5800</v>
-      </c>
-      <c r="J20" t="str">
-        <v>Microsoft</v>
-      </c>
-      <c r="K20" t="str">
-        <v>None</v>
-      </c>
-      <c r="L20" t="str">
-        <v>Master identity and access management system providing Single Sign-On (SSO) and RBAC for all apps.</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="str">
-        <v>Informatica PowerCenter ETL</v>
-      </c>
-      <c r="B21" t="str">
-        <v>Data Architecture</v>
-      </c>
-      <c r="C21" t="str">
-        <v>High</v>
-      </c>
-      <c r="D21">
-        <v>520000</v>
-      </c>
-      <c r="E21" t="str">
-        <v>High Tech Debt</v>
-      </c>
-      <c r="F21" t="str">
-        <v>On-Premises VM</v>
-      </c>
-      <c r="G21" t="str">
-        <v>Informatica Server 9.6, Oracle Repository</v>
-      </c>
-      <c r="H21" t="str">
-        <v>Monolith Heavy</v>
-      </c>
-      <c r="I21">
-        <v>45</v>
-      </c>
-      <c r="J21" t="str">
-        <v>Informatica</v>
-      </c>
-      <c r="K21" t="str">
-        <v>Oracle E-Business Suite 11i, Snowflake Data Warehouse</v>
-      </c>
-      <c r="L21" t="str">
-        <v>On-premises enterprise ETL pipeline with high annual licensing and complex batch dependencies that frequently block data lake updates.</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L21"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L11"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>